<commit_message>
SISU 26.00 korjattu ptoimtuki-parametritaulun virheelliset arvot
</commit_message>
<xml_diff>
--- a/SISU/DOKUM/Lakimuutokset/lakipäivitykset_2026.xlsx
+++ b/SISU/DOKUM/Lakimuutokset/lakipäivitykset_2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sivonenr\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mikrosimulointirepo\Mikrosimulointi\SISU\DOKUM\Lakimuutokset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C59642-6B7E-4D93-81B7-6A6054A0BA3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6B5D6D0-DD4F-492A-87E5-014CD99F103E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29820" yWindow="960" windowWidth="26610" windowHeight="13620" xr2:uid="{1D7543B3-5A4E-4762-90D7-B455325C9A0F}"/>
+    <workbookView xWindow="2100" yWindow="1635" windowWidth="21600" windowHeight="11235" firstSheet="2" activeTab="12" xr2:uid="{1D7543B3-5A4E-4762-90D7-B455325C9A0F}"/>
   </bookViews>
   <sheets>
     <sheet name="Lakimuutokset" sheetId="1" r:id="rId1"/>
@@ -5369,8 +5369,8 @@
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{737DAA11-EC2F-4853-A29F-DFC812235F26}"/>
+    <cellStyle name="Normaali" xfId="0" builtinId="0"/>
     <cellStyle name="Normaali_Taul1" xfId="2" xr:uid="{C259D810-F21D-4435-AC25-5ED9DDA4FD3E}"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -5386,7 +5386,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-teema">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -9143,7 +9143,7 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="J7">
-        <v>0.14000000000000001</v>
+        <v>0.15</v>
       </c>
       <c r="L7">
         <v>1</v>
@@ -9184,7 +9184,7 @@
         <v>0.85</v>
       </c>
       <c r="J8">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="L8">
         <v>1</v>
@@ -9266,7 +9266,7 @@
         <v>0.7</v>
       </c>
       <c r="J10">
-        <v>0.7</v>
+        <v>0.72199999999999998</v>
       </c>
       <c r="L10">
         <v>1</v>
@@ -9308,7 +9308,7 @@
         <v>0.7</v>
       </c>
       <c r="J11">
-        <v>0.7</v>
+        <v>0.72199999999999998</v>
       </c>
       <c r="L11">
         <v>1</v>
@@ -9350,7 +9350,7 @@
         <v>0.63</v>
       </c>
       <c r="J12">
-        <v>0.63</v>
+        <v>0.65</v>
       </c>
       <c r="L12">
         <v>1</v>
@@ -32655,15 +32655,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <DHStatDestinationTaxHTField xmlns="http://schemas.microsoft.com/sharepoint/v3">
@@ -32698,19 +32689,37 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F8E6AA0-8915-4772-8787-C2CA79FE73E4}"/>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B261F99C-B2F2-4374-9EF1-FDFD9752D396}">
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F8E6AA0-8915-4772-8787-C2CA79FE73E4}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="eb806122-3b61-4629-a153-37a7e159d40d"/>
+    <ds:schemaRef ds:uri="c47393e0-5d8b-4651-8fb3-70dce98ec114"/>
+    <ds:schemaRef ds:uri="8adaa443-116c-4e15-911c-c46057ad523c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A2E96A2-4689-4E14-8C5B-EE0A15D2E877}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="eb806122-3b61-4629-a153-37a7e159d40d"/>
@@ -32729,6 +32738,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B261F99C-B2F2-4374-9EF1-FDFD9752D396}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{cf4a4c0d-994f-4f10-923c-4bfde5b4a14e}" enabled="0" method="" siteId="{cf4a4c0d-994f-4f10-923c-4bfde5b4a14e}" removed="1"/>

</xml_diff>